<commit_message>
Improve desktop localization, capture diagnostics, and reflection export
</commit_message>
<xml_diff>
--- a/src/Desktop/resources/import-templates/personal-records.xlsx
+++ b/src/Desktop/resources/import-templates/personal-records.xlsx
@@ -80,6 +80,7 @@
     <col min="8" max="8" width="16" customWidth="1" style="2"/>
     <col min="9" max="9" width="25" customWidth="1" style="2"/>
     <col min="10" max="10" width="45" customWidth="1" style="2"/>
+    <col min="11" max="11" width="20" customWidth="1" style="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -133,6 +134,11 @@
           <t xml:space="preserve">备注</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">进入方式</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" t="inlineStr" s="2">
@@ -185,9 +191,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="K2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="请使用支持的值" error="请选择列表中的值" sqref="E2:E5001">
       <formula1>"通关,未知,离开,放弃,取消,中断,掉线"</formula1>
@@ -458,6 +469,18 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="100" customHeight="1">
+      <c r="A22" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">进入方式 / joined_in_progress</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">正常或开局进入表示从开局进入（false）；中途或中途加入表示中途进入（true）。未知时 Excel 留空，JSON 保留 null；不会自动按正常进入统计。JSON 也可填写布尔值 false 或 true。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>